<commit_message>
Cambios para mejorar score, falta limitar la cantidad de turnos por hora
</commit_message>
<xml_diff>
--- a/Result/CoberturaFinal.xlsx
+++ b/Result/CoberturaFinal.xlsx
@@ -938,13 +938,13 @@
         <v>12</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G16" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1002,13 +1002,13 @@
         <v>380</v>
       </c>
       <c r="E18" t="n">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="F18" t="n">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="G18" t="n">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -1066,13 +1066,13 @@
         <v>416</v>
       </c>
       <c r="E20" t="n">
-        <v>348</v>
+        <v>363</v>
       </c>
       <c r="F20" t="n">
-        <v>348</v>
+        <v>363</v>
       </c>
       <c r="G20" t="n">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -1098,13 +1098,13 @@
         <v>440</v>
       </c>
       <c r="E21" t="n">
-        <v>418</v>
+        <v>373</v>
       </c>
       <c r="F21" t="n">
-        <v>418</v>
+        <v>373</v>
       </c>
       <c r="G21" t="n">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1130,13 +1130,13 @@
         <v>463</v>
       </c>
       <c r="E22" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="F22" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="G22" t="n">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1162,13 +1162,13 @@
         <v>463</v>
       </c>
       <c r="E23" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F23" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G23" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1194,13 +1194,13 @@
         <v>465</v>
       </c>
       <c r="E24" t="n">
-        <v>418</v>
+        <v>394</v>
       </c>
       <c r="F24" t="n">
-        <v>418</v>
+        <v>394</v>
       </c>
       <c r="G24" t="n">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1226,13 +1226,13 @@
         <v>501</v>
       </c>
       <c r="E25" t="n">
-        <v>418</v>
+        <v>394</v>
       </c>
       <c r="F25" t="n">
-        <v>418</v>
+        <v>394</v>
       </c>
       <c r="G25" t="n">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1258,13 +1258,13 @@
         <v>501</v>
       </c>
       <c r="E26" t="n">
-        <v>403</v>
+        <v>358</v>
       </c>
       <c r="F26" t="n">
-        <v>403</v>
+        <v>358</v>
       </c>
       <c r="G26" t="n">
-        <v>98</v>
+        <v>143</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1290,13 +1290,13 @@
         <v>501</v>
       </c>
       <c r="E27" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F27" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G27" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1546,13 +1546,13 @@
         <v>472</v>
       </c>
       <c r="E35" t="n">
-        <v>418</v>
+        <v>406</v>
       </c>
       <c r="F35" t="n">
-        <v>418</v>
+        <v>406</v>
       </c>
       <c r="G35" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -1578,13 +1578,13 @@
         <v>449</v>
       </c>
       <c r="E36" t="n">
-        <v>301</v>
+        <v>370</v>
       </c>
       <c r="F36" t="n">
-        <v>301</v>
+        <v>370</v>
       </c>
       <c r="G36" t="n">
-        <v>148</v>
+        <v>79</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -1674,13 +1674,13 @@
         <v>85</v>
       </c>
       <c r="E39" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="F39" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="G39" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -1706,13 +1706,13 @@
         <v>60</v>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G40" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -1738,13 +1738,13 @@
         <v>37</v>
       </c>
       <c r="E41" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G41" t="n">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -1770,13 +1770,13 @@
         <v>37</v>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G42" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -1802,13 +1802,13 @@
         <v>37</v>
       </c>
       <c r="E43" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G43" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -2474,13 +2474,13 @@
         <v>11</v>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F64" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G64" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -2602,16 +2602,16 @@
         <v>388</v>
       </c>
       <c r="E68" t="n">
-        <v>418</v>
+        <v>373</v>
       </c>
       <c r="F68" t="n">
-        <v>418</v>
+        <v>373</v>
       </c>
       <c r="G68" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H68" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -2634,16 +2634,16 @@
         <v>407</v>
       </c>
       <c r="E69" t="n">
-        <v>418</v>
+        <v>373</v>
       </c>
       <c r="F69" t="n">
-        <v>418</v>
+        <v>373</v>
       </c>
       <c r="G69" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="H69" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -2666,13 +2666,13 @@
         <v>422</v>
       </c>
       <c r="E70" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="F70" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="G70" t="n">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="H70" t="n">
         <v>0</v>
@@ -2698,13 +2698,13 @@
         <v>423</v>
       </c>
       <c r="E71" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F71" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G71" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="H71" t="n">
         <v>0</v>
@@ -2730,13 +2730,13 @@
         <v>427</v>
       </c>
       <c r="E72" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="F72" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="G72" t="n">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="H72" t="n">
         <v>0</v>
@@ -2762,13 +2762,13 @@
         <v>457</v>
       </c>
       <c r="E73" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="F73" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="G73" t="n">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="H73" t="n">
         <v>0</v>
@@ -2794,13 +2794,13 @@
         <v>457</v>
       </c>
       <c r="E74" t="n">
-        <v>403</v>
+        <v>358</v>
       </c>
       <c r="F74" t="n">
-        <v>403</v>
+        <v>358</v>
       </c>
       <c r="G74" t="n">
-        <v>54</v>
+        <v>99</v>
       </c>
       <c r="H74" t="n">
         <v>0</v>
@@ -2826,13 +2826,13 @@
         <v>457</v>
       </c>
       <c r="E75" t="n">
-        <v>418</v>
+        <v>397</v>
       </c>
       <c r="F75" t="n">
-        <v>418</v>
+        <v>397</v>
       </c>
       <c r="G75" t="n">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="H75" t="n">
         <v>0</v>
@@ -2858,13 +2858,13 @@
         <v>458</v>
       </c>
       <c r="E76" t="n">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="F76" t="n">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="G76" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="H76" t="n">
         <v>0</v>
@@ -2890,13 +2890,13 @@
         <v>458</v>
       </c>
       <c r="E77" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F77" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G77" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="H77" t="n">
         <v>0</v>
@@ -2922,13 +2922,13 @@
         <v>455</v>
       </c>
       <c r="E78" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F78" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G78" t="n">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="H78" t="n">
         <v>0</v>
@@ -3082,13 +3082,13 @@
         <v>427</v>
       </c>
       <c r="E83" t="n">
-        <v>416</v>
+        <v>407</v>
       </c>
       <c r="F83" t="n">
-        <v>416</v>
+        <v>407</v>
       </c>
       <c r="G83" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="H83" t="n">
         <v>0</v>
@@ -3114,13 +3114,13 @@
         <v>402</v>
       </c>
       <c r="E84" t="n">
-        <v>290</v>
+        <v>371</v>
       </c>
       <c r="F84" t="n">
-        <v>290</v>
+        <v>371</v>
       </c>
       <c r="G84" t="n">
-        <v>112</v>
+        <v>31</v>
       </c>
       <c r="H84" t="n">
         <v>0</v>
@@ -3210,13 +3210,13 @@
         <v>69</v>
       </c>
       <c r="E87" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F87" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G87" t="n">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="H87" t="n">
         <v>0</v>
@@ -3242,13 +3242,13 @@
         <v>48</v>
       </c>
       <c r="E88" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F88" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G88" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="H88" t="n">
         <v>0</v>
@@ -3274,13 +3274,13 @@
         <v>34</v>
       </c>
       <c r="E89" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F89" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G89" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="H89" t="n">
         <v>0</v>
@@ -3306,13 +3306,13 @@
         <v>34</v>
       </c>
       <c r="E90" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F90" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G90" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="H90" t="n">
         <v>0</v>
@@ -3338,13 +3338,13 @@
         <v>32</v>
       </c>
       <c r="E91" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F91" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G91" t="n">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="H91" t="n">
         <v>0</v>
@@ -4074,13 +4074,13 @@
         <v>319</v>
       </c>
       <c r="E114" t="n">
-        <v>213</v>
+        <v>188</v>
       </c>
       <c r="F114" t="n">
-        <v>213</v>
+        <v>188</v>
       </c>
       <c r="G114" t="n">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="H114" t="n">
         <v>0</v>
@@ -4106,13 +4106,13 @@
         <v>336</v>
       </c>
       <c r="E115" t="n">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="F115" t="n">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="G115" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H115" t="n">
         <v>0</v>
@@ -4138,16 +4138,16 @@
         <v>347</v>
       </c>
       <c r="E116" t="n">
-        <v>411</v>
+        <v>347</v>
       </c>
       <c r="F116" t="n">
-        <v>411</v>
+        <v>347</v>
       </c>
       <c r="G116" t="n">
         <v>0</v>
       </c>
       <c r="H116" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
@@ -4170,16 +4170,16 @@
         <v>364</v>
       </c>
       <c r="E117" t="n">
-        <v>411</v>
+        <v>364</v>
       </c>
       <c r="F117" t="n">
-        <v>411</v>
+        <v>364</v>
       </c>
       <c r="G117" t="n">
         <v>0</v>
       </c>
       <c r="H117" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
@@ -4202,16 +4202,16 @@
         <v>385</v>
       </c>
       <c r="E118" t="n">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="F118" t="n">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="G118" t="n">
         <v>0</v>
       </c>
       <c r="H118" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
@@ -4266,13 +4266,13 @@
         <v>389</v>
       </c>
       <c r="E120" t="n">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="F120" t="n">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="G120" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H120" t="n">
         <v>0</v>
@@ -4298,13 +4298,13 @@
         <v>413</v>
       </c>
       <c r="E121" t="n">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F121" t="n">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="G121" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H121" t="n">
         <v>0</v>
@@ -4330,13 +4330,13 @@
         <v>411</v>
       </c>
       <c r="E122" t="n">
-        <v>396</v>
+        <v>358</v>
       </c>
       <c r="F122" t="n">
-        <v>396</v>
+        <v>358</v>
       </c>
       <c r="G122" t="n">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="H122" t="n">
         <v>0</v>
@@ -4362,13 +4362,13 @@
         <v>411</v>
       </c>
       <c r="E123" t="n">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="F123" t="n">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="G123" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H123" t="n">
         <v>0</v>
@@ -4394,13 +4394,13 @@
         <v>413</v>
       </c>
       <c r="E124" t="n">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="F124" t="n">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="G124" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H124" t="n">
         <v>0</v>
@@ -4426,13 +4426,13 @@
         <v>413</v>
       </c>
       <c r="E125" t="n">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="F125" t="n">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="G125" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H125" t="n">
         <v>0</v>
@@ -4554,13 +4554,13 @@
         <v>409</v>
       </c>
       <c r="E129" t="n">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="F129" t="n">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="G129" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H129" t="n">
         <v>0</v>
@@ -4650,13 +4650,13 @@
         <v>359</v>
       </c>
       <c r="E132" t="n">
-        <v>280</v>
+        <v>359</v>
       </c>
       <c r="F132" t="n">
-        <v>280</v>
+        <v>359</v>
       </c>
       <c r="G132" t="n">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="H132" t="n">
         <v>0</v>
@@ -4746,13 +4746,13 @@
         <v>66</v>
       </c>
       <c r="E135" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="F135" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="G135" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="H135" t="n">
         <v>0</v>
@@ -4778,13 +4778,13 @@
         <v>48</v>
       </c>
       <c r="E136" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="F136" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="G136" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="H136" t="n">
         <v>0</v>
@@ -4810,13 +4810,13 @@
         <v>30</v>
       </c>
       <c r="E137" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F137" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G137" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H137" t="n">
         <v>0</v>
@@ -4842,13 +4842,13 @@
         <v>29</v>
       </c>
       <c r="E138" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F138" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="G138" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="H138" t="n">
         <v>0</v>
@@ -4874,13 +4874,13 @@
         <v>27</v>
       </c>
       <c r="E139" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F139" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="G139" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="H139" t="n">
         <v>0</v>
@@ -5546,13 +5546,13 @@
         <v>7</v>
       </c>
       <c r="E160" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F160" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G160" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H160" t="n">
         <v>0</v>
@@ -5610,13 +5610,13 @@
         <v>362</v>
       </c>
       <c r="E162" t="n">
-        <v>207</v>
+        <v>252</v>
       </c>
       <c r="F162" t="n">
-        <v>207</v>
+        <v>252</v>
       </c>
       <c r="G162" t="n">
-        <v>155</v>
+        <v>110</v>
       </c>
       <c r="H162" t="n">
         <v>0</v>
@@ -5674,16 +5674,16 @@
         <v>391</v>
       </c>
       <c r="E164" t="n">
-        <v>418</v>
+        <v>356</v>
       </c>
       <c r="F164" t="n">
-        <v>418</v>
+        <v>356</v>
       </c>
       <c r="G164" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H164" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165">
@@ -5706,16 +5706,16 @@
         <v>408</v>
       </c>
       <c r="E165" t="n">
-        <v>418</v>
+        <v>376</v>
       </c>
       <c r="F165" t="n">
-        <v>418</v>
+        <v>376</v>
       </c>
       <c r="G165" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="H165" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166">
@@ -5738,13 +5738,13 @@
         <v>428</v>
       </c>
       <c r="E166" t="n">
-        <v>418</v>
+        <v>391</v>
       </c>
       <c r="F166" t="n">
-        <v>418</v>
+        <v>391</v>
       </c>
       <c r="G166" t="n">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="H166" t="n">
         <v>0</v>
@@ -5770,13 +5770,13 @@
         <v>428</v>
       </c>
       <c r="E167" t="n">
-        <v>418</v>
+        <v>406</v>
       </c>
       <c r="F167" t="n">
-        <v>418</v>
+        <v>406</v>
       </c>
       <c r="G167" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="H167" t="n">
         <v>0</v>
@@ -5802,13 +5802,13 @@
         <v>429</v>
       </c>
       <c r="E168" t="n">
-        <v>418</v>
+        <v>391</v>
       </c>
       <c r="F168" t="n">
-        <v>418</v>
+        <v>391</v>
       </c>
       <c r="G168" t="n">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="H168" t="n">
         <v>0</v>
@@ -5834,13 +5834,13 @@
         <v>453</v>
       </c>
       <c r="E169" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F169" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G169" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="H169" t="n">
         <v>0</v>
@@ -5866,13 +5866,13 @@
         <v>454</v>
       </c>
       <c r="E170" t="n">
-        <v>403</v>
+        <v>356</v>
       </c>
       <c r="F170" t="n">
-        <v>403</v>
+        <v>356</v>
       </c>
       <c r="G170" t="n">
-        <v>51</v>
+        <v>98</v>
       </c>
       <c r="H170" t="n">
         <v>0</v>
@@ -5898,13 +5898,13 @@
         <v>454</v>
       </c>
       <c r="E171" t="n">
-        <v>418</v>
+        <v>371</v>
       </c>
       <c r="F171" t="n">
-        <v>418</v>
+        <v>371</v>
       </c>
       <c r="G171" t="n">
-        <v>36</v>
+        <v>83</v>
       </c>
       <c r="H171" t="n">
         <v>0</v>
@@ -5962,13 +5962,13 @@
         <v>454</v>
       </c>
       <c r="E173" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F173" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G173" t="n">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="H173" t="n">
         <v>0</v>
@@ -5994,13 +5994,13 @@
         <v>451</v>
       </c>
       <c r="E174" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F174" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G174" t="n">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="H174" t="n">
         <v>0</v>
@@ -6154,13 +6154,13 @@
         <v>430</v>
       </c>
       <c r="E179" t="n">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="F179" t="n">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="G179" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="H179" t="n">
         <v>0</v>
@@ -6186,13 +6186,13 @@
         <v>390</v>
       </c>
       <c r="E180" t="n">
-        <v>286</v>
+        <v>318</v>
       </c>
       <c r="F180" t="n">
-        <v>286</v>
+        <v>318</v>
       </c>
       <c r="G180" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="H180" t="n">
         <v>0</v>
@@ -6282,13 +6282,13 @@
         <v>62</v>
       </c>
       <c r="E183" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="F183" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="G183" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="H183" t="n">
         <v>0</v>
@@ -6314,13 +6314,13 @@
         <v>45</v>
       </c>
       <c r="E184" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="F184" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="G184" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="H184" t="n">
         <v>0</v>
@@ -6346,13 +6346,13 @@
         <v>27</v>
       </c>
       <c r="E185" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F185" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="G185" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H185" t="n">
         <v>0</v>
@@ -6378,13 +6378,13 @@
         <v>27</v>
       </c>
       <c r="E186" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F186" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G186" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="H186" t="n">
         <v>0</v>
@@ -6410,13 +6410,13 @@
         <v>26</v>
       </c>
       <c r="E187" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F187" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G187" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="H187" t="n">
         <v>0</v>
@@ -7082,13 +7082,13 @@
         <v>6</v>
       </c>
       <c r="E208" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F208" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G208" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H208" t="n">
         <v>0</v>
@@ -7146,13 +7146,13 @@
         <v>367</v>
       </c>
       <c r="E210" t="n">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="F210" t="n">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="G210" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="H210" t="n">
         <v>0</v>
@@ -7210,16 +7210,16 @@
         <v>402</v>
       </c>
       <c r="E212" t="n">
-        <v>418</v>
+        <v>373</v>
       </c>
       <c r="F212" t="n">
-        <v>418</v>
+        <v>373</v>
       </c>
       <c r="G212" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="H212" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="213">
@@ -7242,13 +7242,13 @@
         <v>422</v>
       </c>
       <c r="E213" t="n">
-        <v>418</v>
+        <v>373</v>
       </c>
       <c r="F213" t="n">
-        <v>418</v>
+        <v>373</v>
       </c>
       <c r="G213" t="n">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="H213" t="n">
         <v>0</v>
@@ -7274,13 +7274,13 @@
         <v>438</v>
       </c>
       <c r="E214" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="F214" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="G214" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H214" t="n">
         <v>0</v>
@@ -7306,13 +7306,13 @@
         <v>438</v>
       </c>
       <c r="E215" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="F215" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="G215" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H215" t="n">
         <v>0</v>
@@ -7338,13 +7338,13 @@
         <v>440</v>
       </c>
       <c r="E216" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="F216" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="G216" t="n">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="H216" t="n">
         <v>0</v>
@@ -7402,13 +7402,13 @@
         <v>472</v>
       </c>
       <c r="E218" t="n">
-        <v>412</v>
+        <v>318</v>
       </c>
       <c r="F218" t="n">
-        <v>412</v>
+        <v>318</v>
       </c>
       <c r="G218" t="n">
-        <v>60</v>
+        <v>154</v>
       </c>
       <c r="H218" t="n">
         <v>0</v>
@@ -7434,13 +7434,13 @@
         <v>472</v>
       </c>
       <c r="E219" t="n">
-        <v>418</v>
+        <v>318</v>
       </c>
       <c r="F219" t="n">
-        <v>418</v>
+        <v>318</v>
       </c>
       <c r="G219" t="n">
-        <v>54</v>
+        <v>154</v>
       </c>
       <c r="H219" t="n">
         <v>0</v>
@@ -7466,13 +7466,13 @@
         <v>473</v>
       </c>
       <c r="E220" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="F220" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="G220" t="n">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="H220" t="n">
         <v>0</v>
@@ -7498,13 +7498,13 @@
         <v>473</v>
       </c>
       <c r="E221" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="F221" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="G221" t="n">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="H221" t="n">
         <v>0</v>
@@ -7530,13 +7530,13 @@
         <v>472</v>
       </c>
       <c r="E222" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F222" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G222" t="n">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="H222" t="n">
         <v>0</v>
@@ -7562,13 +7562,13 @@
         <v>471</v>
       </c>
       <c r="E223" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F223" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G223" t="n">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="H223" t="n">
         <v>0</v>
@@ -7594,13 +7594,13 @@
         <v>468</v>
       </c>
       <c r="E224" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F224" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G224" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H224" t="n">
         <v>0</v>
@@ -7690,13 +7690,13 @@
         <v>431</v>
       </c>
       <c r="E227" t="n">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="F227" t="n">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="G227" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="H227" t="n">
         <v>0</v>
@@ -7818,13 +7818,13 @@
         <v>73</v>
       </c>
       <c r="E231" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F231" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G231" t="n">
-        <v>73</v>
+        <v>28</v>
       </c>
       <c r="H231" t="n">
         <v>0</v>
@@ -7850,13 +7850,13 @@
         <v>52</v>
       </c>
       <c r="E232" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F232" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G232" t="n">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="H232" t="n">
         <v>0</v>
@@ -7882,13 +7882,13 @@
         <v>35</v>
       </c>
       <c r="E233" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F233" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G233" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="H233" t="n">
         <v>0</v>
@@ -7914,13 +7914,13 @@
         <v>35</v>
       </c>
       <c r="E234" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F234" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G234" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="H234" t="n">
         <v>0</v>
@@ -7946,13 +7946,13 @@
         <v>34</v>
       </c>
       <c r="E235" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F235" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G235" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="H235" t="n">
         <v>0</v>
@@ -8685,10 +8685,10 @@
         <v>204</v>
       </c>
       <c r="F258" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G258" t="n">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="H258" t="n">
         <v>0</v>
@@ -8714,13 +8714,13 @@
         <v>204</v>
       </c>
       <c r="E259" t="n">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="F259" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G259" t="n">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="H259" t="n">
         <v>0</v>
@@ -8749,10 +8749,10 @@
         <v>208</v>
       </c>
       <c r="F260" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G260" t="n">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="H260" t="n">
         <v>0</v>
@@ -8781,10 +8781,10 @@
         <v>208</v>
       </c>
       <c r="F261" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G261" t="n">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="H261" t="n">
         <v>0</v>
@@ -8813,10 +8813,10 @@
         <v>208</v>
       </c>
       <c r="F262" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G262" t="n">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="H262" t="n">
         <v>0</v>
@@ -8845,10 +8845,10 @@
         <v>208</v>
       </c>
       <c r="F263" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G263" t="n">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="H263" t="n">
         <v>0</v>
@@ -8877,10 +8877,10 @@
         <v>208</v>
       </c>
       <c r="F264" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G264" t="n">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="H264" t="n">
         <v>0</v>
@@ -8909,10 +8909,10 @@
         <v>208</v>
       </c>
       <c r="F265" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G265" t="n">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="H265" t="n">
         <v>0</v>
@@ -8941,10 +8941,10 @@
         <v>208</v>
       </c>
       <c r="F266" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G266" t="n">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="H266" t="n">
         <v>0</v>
@@ -8973,10 +8973,10 @@
         <v>208</v>
       </c>
       <c r="F267" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G267" t="n">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="H267" t="n">
         <v>0</v>
@@ -9005,10 +9005,10 @@
         <v>208</v>
       </c>
       <c r="F268" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G268" t="n">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="H268" t="n">
         <v>0</v>
@@ -9037,10 +9037,10 @@
         <v>208</v>
       </c>
       <c r="F269" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G269" t="n">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="H269" t="n">
         <v>0</v>
@@ -9069,10 +9069,10 @@
         <v>205</v>
       </c>
       <c r="F270" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G270" t="n">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="H270" t="n">
         <v>0</v>
@@ -9101,10 +9101,10 @@
         <v>205</v>
       </c>
       <c r="F271" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G271" t="n">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="H271" t="n">
         <v>0</v>
@@ -9133,10 +9133,10 @@
         <v>201</v>
       </c>
       <c r="F272" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G272" t="n">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="H272" t="n">
         <v>0</v>
@@ -9165,10 +9165,10 @@
         <v>201</v>
       </c>
       <c r="F273" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G273" t="n">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="H273" t="n">
         <v>0</v>
@@ -9197,10 +9197,10 @@
         <v>198</v>
       </c>
       <c r="F274" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G274" t="n">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="H274" t="n">
         <v>0</v>
@@ -9229,10 +9229,10 @@
         <v>198</v>
       </c>
       <c r="F275" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G275" t="n">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="H275" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Reestructuración pra inlcuir mas horarios de menos horas, principalmente <7
</commit_message>
<xml_diff>
--- a/Result/CoberturaFinal.xlsx
+++ b/Result/CoberturaFinal.xlsx
@@ -938,13 +938,13 @@
         <v>12</v>
       </c>
       <c r="E16" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1002,13 +1002,13 @@
         <v>380</v>
       </c>
       <c r="E18" t="n">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="F18" t="n">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="G18" t="n">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -1034,13 +1034,13 @@
         <v>400</v>
       </c>
       <c r="E19" t="n">
-        <v>318</v>
+        <v>279</v>
       </c>
       <c r="F19" t="n">
-        <v>318</v>
+        <v>279</v>
       </c>
       <c r="G19" t="n">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -1066,13 +1066,13 @@
         <v>416</v>
       </c>
       <c r="E20" t="n">
-        <v>343</v>
+        <v>363</v>
       </c>
       <c r="F20" t="n">
-        <v>343</v>
+        <v>363</v>
       </c>
       <c r="G20" t="n">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -1098,13 +1098,13 @@
         <v>440</v>
       </c>
       <c r="E21" t="n">
-        <v>358</v>
+        <v>393</v>
       </c>
       <c r="F21" t="n">
-        <v>358</v>
+        <v>393</v>
       </c>
       <c r="G21" t="n">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1130,13 +1130,13 @@
         <v>463</v>
       </c>
       <c r="E22" t="n">
-        <v>388</v>
+        <v>403</v>
       </c>
       <c r="F22" t="n">
-        <v>388</v>
+        <v>403</v>
       </c>
       <c r="G22" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1162,13 +1162,13 @@
         <v>463</v>
       </c>
       <c r="E23" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F23" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G23" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1194,13 +1194,13 @@
         <v>465</v>
       </c>
       <c r="E24" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F24" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G24" t="n">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1258,13 +1258,13 @@
         <v>501</v>
       </c>
       <c r="E26" t="n">
-        <v>364</v>
+        <v>343</v>
       </c>
       <c r="F26" t="n">
-        <v>364</v>
+        <v>343</v>
       </c>
       <c r="G26" t="n">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1290,13 +1290,13 @@
         <v>501</v>
       </c>
       <c r="E27" t="n">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="F27" t="n">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="G27" t="n">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1322,13 +1322,13 @@
         <v>502</v>
       </c>
       <c r="E28" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="F28" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="G28" t="n">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -1546,13 +1546,13 @@
         <v>472</v>
       </c>
       <c r="E35" t="n">
-        <v>406</v>
+        <v>415</v>
       </c>
       <c r="F35" t="n">
-        <v>406</v>
+        <v>415</v>
       </c>
       <c r="G35" t="n">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -1578,13 +1578,13 @@
         <v>449</v>
       </c>
       <c r="E36" t="n">
-        <v>370</v>
+        <v>325</v>
       </c>
       <c r="F36" t="n">
-        <v>370</v>
+        <v>325</v>
       </c>
       <c r="G36" t="n">
-        <v>79</v>
+        <v>124</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -1674,13 +1674,13 @@
         <v>85</v>
       </c>
       <c r="E39" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="F39" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="G39" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -1706,13 +1706,13 @@
         <v>60</v>
       </c>
       <c r="E40" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="F40" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -1738,13 +1738,13 @@
         <v>37</v>
       </c>
       <c r="E41" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F41" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="G41" t="n">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -1770,13 +1770,13 @@
         <v>37</v>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G42" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -1802,13 +1802,13 @@
         <v>37</v>
       </c>
       <c r="E43" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G43" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -2474,13 +2474,13 @@
         <v>11</v>
       </c>
       <c r="E64" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="F64" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G64" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -2538,13 +2538,13 @@
         <v>360</v>
       </c>
       <c r="E66" t="n">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="F66" t="n">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="G66" t="n">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
@@ -2570,13 +2570,13 @@
         <v>374</v>
       </c>
       <c r="E67" t="n">
-        <v>337</v>
+        <v>287</v>
       </c>
       <c r="F67" t="n">
-        <v>337</v>
+        <v>287</v>
       </c>
       <c r="G67" t="n">
-        <v>37</v>
+        <v>87</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -2602,13 +2602,13 @@
         <v>388</v>
       </c>
       <c r="E68" t="n">
-        <v>355</v>
+        <v>382</v>
       </c>
       <c r="F68" t="n">
-        <v>355</v>
+        <v>382</v>
       </c>
       <c r="G68" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
@@ -2634,13 +2634,13 @@
         <v>407</v>
       </c>
       <c r="E69" t="n">
-        <v>370</v>
+        <v>407</v>
       </c>
       <c r="F69" t="n">
-        <v>370</v>
+        <v>407</v>
       </c>
       <c r="G69" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
@@ -2666,13 +2666,13 @@
         <v>422</v>
       </c>
       <c r="E70" t="n">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="F70" t="n">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="G70" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H70" t="n">
         <v>0</v>
@@ -2698,13 +2698,13 @@
         <v>423</v>
       </c>
       <c r="E71" t="n">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="F71" t="n">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="G71" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="H71" t="n">
         <v>0</v>
@@ -2730,13 +2730,13 @@
         <v>427</v>
       </c>
       <c r="E72" t="n">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="F72" t="n">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="G72" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H72" t="n">
         <v>0</v>
@@ -2762,13 +2762,13 @@
         <v>457</v>
       </c>
       <c r="E73" t="n">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="F73" t="n">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="G73" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="H73" t="n">
         <v>0</v>
@@ -2794,13 +2794,13 @@
         <v>457</v>
       </c>
       <c r="E74" t="n">
-        <v>343</v>
+        <v>328</v>
       </c>
       <c r="F74" t="n">
-        <v>343</v>
+        <v>328</v>
       </c>
       <c r="G74" t="n">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="H74" t="n">
         <v>0</v>
@@ -2826,13 +2826,13 @@
         <v>457</v>
       </c>
       <c r="E75" t="n">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="F75" t="n">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="G75" t="n">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="H75" t="n">
         <v>0</v>
@@ -2858,13 +2858,13 @@
         <v>458</v>
       </c>
       <c r="E76" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="F76" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="G76" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="H76" t="n">
         <v>0</v>
@@ -3082,13 +3082,13 @@
         <v>427</v>
       </c>
       <c r="E83" t="n">
-        <v>407</v>
+        <v>416</v>
       </c>
       <c r="F83" t="n">
-        <v>407</v>
+        <v>416</v>
       </c>
       <c r="G83" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="H83" t="n">
         <v>0</v>
@@ -3114,13 +3114,13 @@
         <v>402</v>
       </c>
       <c r="E84" t="n">
-        <v>371</v>
+        <v>326</v>
       </c>
       <c r="F84" t="n">
-        <v>371</v>
+        <v>326</v>
       </c>
       <c r="G84" t="n">
-        <v>31</v>
+        <v>76</v>
       </c>
       <c r="H84" t="n">
         <v>0</v>
@@ -3210,13 +3210,13 @@
         <v>69</v>
       </c>
       <c r="E87" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="F87" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="G87" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="H87" t="n">
         <v>0</v>
@@ -3242,13 +3242,13 @@
         <v>48</v>
       </c>
       <c r="E88" t="n">
-        <v>48</v>
+        <v>11</v>
       </c>
       <c r="F88" t="n">
-        <v>48</v>
+        <v>11</v>
       </c>
       <c r="G88" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="H88" t="n">
         <v>0</v>
@@ -3274,13 +3274,13 @@
         <v>34</v>
       </c>
       <c r="E89" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F89" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="G89" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H89" t="n">
         <v>0</v>
@@ -3306,13 +3306,13 @@
         <v>34</v>
       </c>
       <c r="E90" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F90" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G90" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="H90" t="n">
         <v>0</v>
@@ -3338,13 +3338,13 @@
         <v>32</v>
       </c>
       <c r="E91" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F91" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G91" t="n">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="H91" t="n">
         <v>0</v>
@@ -4074,13 +4074,13 @@
         <v>319</v>
       </c>
       <c r="E114" t="n">
-        <v>188</v>
+        <v>213</v>
       </c>
       <c r="F114" t="n">
-        <v>188</v>
+        <v>213</v>
       </c>
       <c r="G114" t="n">
-        <v>131</v>
+        <v>106</v>
       </c>
       <c r="H114" t="n">
         <v>0</v>
@@ -4106,13 +4106,13 @@
         <v>336</v>
       </c>
       <c r="E115" t="n">
-        <v>336</v>
+        <v>310</v>
       </c>
       <c r="F115" t="n">
-        <v>336</v>
+        <v>310</v>
       </c>
       <c r="G115" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="H115" t="n">
         <v>0</v>
@@ -4330,13 +4330,13 @@
         <v>411</v>
       </c>
       <c r="E122" t="n">
-        <v>373</v>
+        <v>338</v>
       </c>
       <c r="F122" t="n">
-        <v>373</v>
+        <v>338</v>
       </c>
       <c r="G122" t="n">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="H122" t="n">
         <v>0</v>
@@ -4362,13 +4362,13 @@
         <v>411</v>
       </c>
       <c r="E123" t="n">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="F123" t="n">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="G123" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="H123" t="n">
         <v>0</v>
@@ -4394,13 +4394,13 @@
         <v>413</v>
       </c>
       <c r="E124" t="n">
-        <v>402</v>
+        <v>413</v>
       </c>
       <c r="F124" t="n">
-        <v>402</v>
+        <v>413</v>
       </c>
       <c r="G124" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H124" t="n">
         <v>0</v>
@@ -4426,13 +4426,13 @@
         <v>413</v>
       </c>
       <c r="E125" t="n">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="F125" t="n">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="G125" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H125" t="n">
         <v>0</v>
@@ -4650,13 +4650,13 @@
         <v>359</v>
       </c>
       <c r="E132" t="n">
-        <v>359</v>
+        <v>300</v>
       </c>
       <c r="F132" t="n">
-        <v>359</v>
+        <v>300</v>
       </c>
       <c r="G132" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="H132" t="n">
         <v>0</v>
@@ -4842,13 +4842,13 @@
         <v>29</v>
       </c>
       <c r="E138" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F138" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G138" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H138" t="n">
         <v>0</v>
@@ -4874,13 +4874,13 @@
         <v>27</v>
       </c>
       <c r="E139" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F139" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="G139" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H139" t="n">
         <v>0</v>
@@ -5546,13 +5546,13 @@
         <v>7</v>
       </c>
       <c r="E160" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F160" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G160" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H160" t="n">
         <v>0</v>
@@ -5610,13 +5610,13 @@
         <v>362</v>
       </c>
       <c r="E162" t="n">
-        <v>267</v>
+        <v>205</v>
       </c>
       <c r="F162" t="n">
-        <v>267</v>
+        <v>205</v>
       </c>
       <c r="G162" t="n">
-        <v>95</v>
+        <v>157</v>
       </c>
       <c r="H162" t="n">
         <v>0</v>
@@ -5642,13 +5642,13 @@
         <v>376</v>
       </c>
       <c r="E163" t="n">
-        <v>344</v>
+        <v>325</v>
       </c>
       <c r="F163" t="n">
-        <v>344</v>
+        <v>325</v>
       </c>
       <c r="G163" t="n">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H163" t="n">
         <v>0</v>
@@ -5674,13 +5674,13 @@
         <v>391</v>
       </c>
       <c r="E164" t="n">
-        <v>374</v>
+        <v>356</v>
       </c>
       <c r="F164" t="n">
-        <v>374</v>
+        <v>356</v>
       </c>
       <c r="G164" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="H164" t="n">
         <v>0</v>
@@ -5706,13 +5706,13 @@
         <v>408</v>
       </c>
       <c r="E165" t="n">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="F165" t="n">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="G165" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="H165" t="n">
         <v>0</v>
@@ -5738,13 +5738,13 @@
         <v>428</v>
       </c>
       <c r="E166" t="n">
-        <v>391</v>
+        <v>401</v>
       </c>
       <c r="F166" t="n">
-        <v>391</v>
+        <v>401</v>
       </c>
       <c r="G166" t="n">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="H166" t="n">
         <v>0</v>
@@ -5770,13 +5770,13 @@
         <v>428</v>
       </c>
       <c r="E167" t="n">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="F167" t="n">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="G167" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H167" t="n">
         <v>0</v>
@@ -5802,13 +5802,13 @@
         <v>429</v>
       </c>
       <c r="E168" t="n">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="F168" t="n">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G168" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H168" t="n">
         <v>0</v>
@@ -5834,13 +5834,13 @@
         <v>453</v>
       </c>
       <c r="E169" t="n">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="F169" t="n">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="G169" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H169" t="n">
         <v>0</v>
@@ -5866,13 +5866,13 @@
         <v>454</v>
       </c>
       <c r="E170" t="n">
-        <v>358</v>
+        <v>328</v>
       </c>
       <c r="F170" t="n">
-        <v>358</v>
+        <v>328</v>
       </c>
       <c r="G170" t="n">
-        <v>96</v>
+        <v>126</v>
       </c>
       <c r="H170" t="n">
         <v>0</v>
@@ -5898,13 +5898,13 @@
         <v>454</v>
       </c>
       <c r="E171" t="n">
-        <v>388</v>
+        <v>343</v>
       </c>
       <c r="F171" t="n">
-        <v>388</v>
+        <v>343</v>
       </c>
       <c r="G171" t="n">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="H171" t="n">
         <v>0</v>
@@ -5930,13 +5930,13 @@
         <v>454</v>
       </c>
       <c r="E172" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="F172" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="G172" t="n">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="H172" t="n">
         <v>0</v>
@@ -5962,13 +5962,13 @@
         <v>454</v>
       </c>
       <c r="E173" t="n">
-        <v>388</v>
+        <v>418</v>
       </c>
       <c r="F173" t="n">
-        <v>388</v>
+        <v>418</v>
       </c>
       <c r="G173" t="n">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="H173" t="n">
         <v>0</v>
@@ -5994,13 +5994,13 @@
         <v>451</v>
       </c>
       <c r="E174" t="n">
-        <v>388</v>
+        <v>418</v>
       </c>
       <c r="F174" t="n">
-        <v>388</v>
+        <v>418</v>
       </c>
       <c r="G174" t="n">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="H174" t="n">
         <v>0</v>
@@ -6026,13 +6026,13 @@
         <v>451</v>
       </c>
       <c r="E175" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="F175" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="G175" t="n">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="H175" t="n">
         <v>0</v>
@@ -6154,13 +6154,13 @@
         <v>430</v>
       </c>
       <c r="E179" t="n">
-        <v>418</v>
+        <v>396</v>
       </c>
       <c r="F179" t="n">
-        <v>418</v>
+        <v>396</v>
       </c>
       <c r="G179" t="n">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="H179" t="n">
         <v>0</v>
@@ -6282,13 +6282,13 @@
         <v>62</v>
       </c>
       <c r="E183" t="n">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="F183" t="n">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="G183" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="H183" t="n">
         <v>0</v>
@@ -6314,13 +6314,13 @@
         <v>45</v>
       </c>
       <c r="E184" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F184" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G184" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="H184" t="n">
         <v>0</v>
@@ -6346,13 +6346,13 @@
         <v>27</v>
       </c>
       <c r="E185" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F185" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="G185" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H185" t="n">
         <v>0</v>
@@ -6378,13 +6378,13 @@
         <v>27</v>
       </c>
       <c r="E186" t="n">
+        <v>15</v>
+      </c>
+      <c r="F186" t="n">
+        <v>15</v>
+      </c>
+      <c r="G186" t="n">
         <v>12</v>
-      </c>
-      <c r="F186" t="n">
-        <v>12</v>
-      </c>
-      <c r="G186" t="n">
-        <v>15</v>
       </c>
       <c r="H186" t="n">
         <v>0</v>
@@ -6410,13 +6410,13 @@
         <v>26</v>
       </c>
       <c r="E187" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F187" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G187" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H187" t="n">
         <v>0</v>
@@ -7082,13 +7082,13 @@
         <v>6</v>
       </c>
       <c r="E208" t="n">
+        <v>0</v>
+      </c>
+      <c r="F208" t="n">
+        <v>0</v>
+      </c>
+      <c r="G208" t="n">
         <v>6</v>
-      </c>
-      <c r="F208" t="n">
-        <v>6</v>
-      </c>
-      <c r="G208" t="n">
-        <v>0</v>
       </c>
       <c r="H208" t="n">
         <v>0</v>
@@ -7146,13 +7146,13 @@
         <v>367</v>
       </c>
       <c r="E210" t="n">
-        <v>277</v>
+        <v>187</v>
       </c>
       <c r="F210" t="n">
-        <v>277</v>
+        <v>97</v>
       </c>
       <c r="G210" t="n">
-        <v>90</v>
+        <v>270</v>
       </c>
       <c r="H210" t="n">
         <v>0</v>
@@ -7178,13 +7178,13 @@
         <v>385</v>
       </c>
       <c r="E211" t="n">
-        <v>331</v>
+        <v>286</v>
       </c>
       <c r="F211" t="n">
-        <v>331</v>
+        <v>118</v>
       </c>
       <c r="G211" t="n">
-        <v>54</v>
+        <v>267</v>
       </c>
       <c r="H211" t="n">
         <v>0</v>
@@ -7210,13 +7210,13 @@
         <v>402</v>
       </c>
       <c r="E212" t="n">
-        <v>351</v>
+        <v>376</v>
       </c>
       <c r="F212" t="n">
-        <v>351</v>
+        <v>208</v>
       </c>
       <c r="G212" t="n">
-        <v>51</v>
+        <v>194</v>
       </c>
       <c r="H212" t="n">
         <v>0</v>
@@ -7242,13 +7242,13 @@
         <v>422</v>
       </c>
       <c r="E213" t="n">
-        <v>366</v>
+        <v>406</v>
       </c>
       <c r="F213" t="n">
-        <v>366</v>
+        <v>238</v>
       </c>
       <c r="G213" t="n">
-        <v>56</v>
+        <v>184</v>
       </c>
       <c r="H213" t="n">
         <v>0</v>
@@ -7274,13 +7274,13 @@
         <v>438</v>
       </c>
       <c r="E214" t="n">
-        <v>396</v>
+        <v>406</v>
       </c>
       <c r="F214" t="n">
-        <v>396</v>
+        <v>238</v>
       </c>
       <c r="G214" t="n">
-        <v>42</v>
+        <v>200</v>
       </c>
       <c r="H214" t="n">
         <v>0</v>
@@ -7306,13 +7306,13 @@
         <v>438</v>
       </c>
       <c r="E215" t="n">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="F215" t="n">
-        <v>408</v>
+        <v>238</v>
       </c>
       <c r="G215" t="n">
-        <v>30</v>
+        <v>200</v>
       </c>
       <c r="H215" t="n">
         <v>0</v>
@@ -7338,13 +7338,13 @@
         <v>440</v>
       </c>
       <c r="E216" t="n">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="F216" t="n">
-        <v>408</v>
+        <v>238</v>
       </c>
       <c r="G216" t="n">
-        <v>32</v>
+        <v>202</v>
       </c>
       <c r="H216" t="n">
         <v>0</v>
@@ -7373,10 +7373,10 @@
         <v>418</v>
       </c>
       <c r="F217" t="n">
-        <v>418</v>
+        <v>250</v>
       </c>
       <c r="G217" t="n">
-        <v>54</v>
+        <v>222</v>
       </c>
       <c r="H217" t="n">
         <v>0</v>
@@ -7402,13 +7402,13 @@
         <v>472</v>
       </c>
       <c r="E218" t="n">
-        <v>313</v>
+        <v>363</v>
       </c>
       <c r="F218" t="n">
-        <v>313</v>
+        <v>195</v>
       </c>
       <c r="G218" t="n">
-        <v>159</v>
+        <v>277</v>
       </c>
       <c r="H218" t="n">
         <v>0</v>
@@ -7434,13 +7434,13 @@
         <v>472</v>
       </c>
       <c r="E219" t="n">
-        <v>313</v>
+        <v>405</v>
       </c>
       <c r="F219" t="n">
-        <v>313</v>
+        <v>237</v>
       </c>
       <c r="G219" t="n">
-        <v>159</v>
+        <v>235</v>
       </c>
       <c r="H219" t="n">
         <v>0</v>
@@ -7466,13 +7466,13 @@
         <v>473</v>
       </c>
       <c r="E220" t="n">
-        <v>388</v>
+        <v>418</v>
       </c>
       <c r="F220" t="n">
-        <v>388</v>
+        <v>250</v>
       </c>
       <c r="G220" t="n">
-        <v>85</v>
+        <v>223</v>
       </c>
       <c r="H220" t="n">
         <v>0</v>
@@ -7498,13 +7498,13 @@
         <v>473</v>
       </c>
       <c r="E221" t="n">
-        <v>388</v>
+        <v>418</v>
       </c>
       <c r="F221" t="n">
-        <v>388</v>
+        <v>250</v>
       </c>
       <c r="G221" t="n">
-        <v>85</v>
+        <v>223</v>
       </c>
       <c r="H221" t="n">
         <v>0</v>
@@ -7530,13 +7530,13 @@
         <v>472</v>
       </c>
       <c r="E222" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="F222" t="n">
-        <v>403</v>
+        <v>250</v>
       </c>
       <c r="G222" t="n">
-        <v>69</v>
+        <v>222</v>
       </c>
       <c r="H222" t="n">
         <v>0</v>
@@ -7562,13 +7562,13 @@
         <v>471</v>
       </c>
       <c r="E223" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="F223" t="n">
-        <v>403</v>
+        <v>250</v>
       </c>
       <c r="G223" t="n">
-        <v>68</v>
+        <v>221</v>
       </c>
       <c r="H223" t="n">
         <v>0</v>
@@ -7594,13 +7594,13 @@
         <v>468</v>
       </c>
       <c r="E224" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="F224" t="n">
-        <v>403</v>
+        <v>250</v>
       </c>
       <c r="G224" t="n">
-        <v>65</v>
+        <v>218</v>
       </c>
       <c r="H224" t="n">
         <v>0</v>
@@ -7629,10 +7629,10 @@
         <v>418</v>
       </c>
       <c r="F225" t="n">
-        <v>418</v>
+        <v>250</v>
       </c>
       <c r="G225" t="n">
-        <v>44</v>
+        <v>212</v>
       </c>
       <c r="H225" t="n">
         <v>0</v>
@@ -7661,10 +7661,10 @@
         <v>418</v>
       </c>
       <c r="F226" t="n">
-        <v>418</v>
+        <v>250</v>
       </c>
       <c r="G226" t="n">
-        <v>20</v>
+        <v>188</v>
       </c>
       <c r="H226" t="n">
         <v>0</v>
@@ -7690,13 +7690,13 @@
         <v>431</v>
       </c>
       <c r="E227" t="n">
-        <v>412</v>
+        <v>388</v>
       </c>
       <c r="F227" t="n">
-        <v>412</v>
+        <v>250</v>
       </c>
       <c r="G227" t="n">
-        <v>19</v>
+        <v>181</v>
       </c>
       <c r="H227" t="n">
         <v>0</v>
@@ -7725,10 +7725,10 @@
         <v>216</v>
       </c>
       <c r="F228" t="n">
-        <v>216</v>
+        <v>168</v>
       </c>
       <c r="G228" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="H228" t="n">
         <v>0</v>
@@ -7818,13 +7818,13 @@
         <v>73</v>
       </c>
       <c r="E231" t="n">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="G231" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="H231" t="n">
         <v>0</v>
@@ -7850,13 +7850,13 @@
         <v>52</v>
       </c>
       <c r="E232" t="n">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="F232" t="n">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="G232" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H232" t="n">
         <v>0</v>
@@ -7882,13 +7882,13 @@
         <v>35</v>
       </c>
       <c r="E233" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F233" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G233" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="H233" t="n">
         <v>0</v>
@@ -7914,13 +7914,13 @@
         <v>35</v>
       </c>
       <c r="E234" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F234" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G234" t="n">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="H234" t="n">
         <v>0</v>
@@ -7946,13 +7946,13 @@
         <v>34</v>
       </c>
       <c r="E235" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F235" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G235" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="H235" t="n">
         <v>0</v>
@@ -8685,10 +8685,10 @@
         <v>204</v>
       </c>
       <c r="F258" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="G258" t="n">
-        <v>204</v>
+        <v>60</v>
       </c>
       <c r="H258" t="n">
         <v>0</v>
@@ -8717,10 +8717,10 @@
         <v>204</v>
       </c>
       <c r="F259" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="G259" t="n">
-        <v>204</v>
+        <v>60</v>
       </c>
       <c r="H259" t="n">
         <v>0</v>
@@ -8746,13 +8746,13 @@
         <v>206</v>
       </c>
       <c r="E260" t="n">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F260" t="n">
-        <v>0</v>
+        <v>146</v>
       </c>
       <c r="G260" t="n">
-        <v>206</v>
+        <v>60</v>
       </c>
       <c r="H260" t="n">
         <v>0</v>
@@ -8778,13 +8778,13 @@
         <v>207</v>
       </c>
       <c r="E261" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F261" t="n">
-        <v>0</v>
+        <v>147</v>
       </c>
       <c r="G261" t="n">
-        <v>207</v>
+        <v>60</v>
       </c>
       <c r="H261" t="n">
         <v>0</v>
@@ -8813,10 +8813,10 @@
         <v>208</v>
       </c>
       <c r="F262" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="G262" t="n">
-        <v>208</v>
+        <v>60</v>
       </c>
       <c r="H262" t="n">
         <v>0</v>
@@ -8845,10 +8845,10 @@
         <v>208</v>
       </c>
       <c r="F263" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="G263" t="n">
-        <v>208</v>
+        <v>60</v>
       </c>
       <c r="H263" t="n">
         <v>0</v>
@@ -8874,13 +8874,13 @@
         <v>209</v>
       </c>
       <c r="E264" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F264" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="G264" t="n">
-        <v>209</v>
+        <v>60</v>
       </c>
       <c r="H264" t="n">
         <v>0</v>
@@ -8906,13 +8906,13 @@
         <v>209</v>
       </c>
       <c r="E265" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F265" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="G265" t="n">
-        <v>209</v>
+        <v>60</v>
       </c>
       <c r="H265" t="n">
         <v>0</v>
@@ -8938,13 +8938,13 @@
         <v>209</v>
       </c>
       <c r="E266" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F266" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="G266" t="n">
-        <v>209</v>
+        <v>60</v>
       </c>
       <c r="H266" t="n">
         <v>0</v>
@@ -8970,13 +8970,13 @@
         <v>209</v>
       </c>
       <c r="E267" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F267" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="G267" t="n">
-        <v>209</v>
+        <v>60</v>
       </c>
       <c r="H267" t="n">
         <v>0</v>
@@ -9002,13 +9002,13 @@
         <v>209</v>
       </c>
       <c r="E268" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F268" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="G268" t="n">
-        <v>209</v>
+        <v>60</v>
       </c>
       <c r="H268" t="n">
         <v>0</v>
@@ -9037,10 +9037,10 @@
         <v>208</v>
       </c>
       <c r="F269" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="G269" t="n">
-        <v>208</v>
+        <v>60</v>
       </c>
       <c r="H269" t="n">
         <v>0</v>
@@ -9069,10 +9069,10 @@
         <v>205</v>
       </c>
       <c r="F270" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="G270" t="n">
-        <v>205</v>
+        <v>60</v>
       </c>
       <c r="H270" t="n">
         <v>0</v>
@@ -9101,10 +9101,10 @@
         <v>205</v>
       </c>
       <c r="F271" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="G271" t="n">
-        <v>205</v>
+        <v>60</v>
       </c>
       <c r="H271" t="n">
         <v>0</v>
@@ -9133,10 +9133,10 @@
         <v>201</v>
       </c>
       <c r="F272" t="n">
-        <v>0</v>
+        <v>141</v>
       </c>
       <c r="G272" t="n">
-        <v>201</v>
+        <v>60</v>
       </c>
       <c r="H272" t="n">
         <v>0</v>
@@ -9165,10 +9165,10 @@
         <v>201</v>
       </c>
       <c r="F273" t="n">
-        <v>0</v>
+        <v>141</v>
       </c>
       <c r="G273" t="n">
-        <v>201</v>
+        <v>60</v>
       </c>
       <c r="H273" t="n">
         <v>0</v>
@@ -9197,10 +9197,10 @@
         <v>198</v>
       </c>
       <c r="F274" t="n">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="G274" t="n">
-        <v>198</v>
+        <v>60</v>
       </c>
       <c r="H274" t="n">
         <v>0</v>
@@ -9229,10 +9229,10 @@
         <v>198</v>
       </c>
       <c r="F275" t="n">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="G275" t="n">
-        <v>198</v>
+        <v>60</v>
       </c>
       <c r="H275" t="n">
         <v>0</v>
@@ -10221,10 +10221,10 @@
         <v>41</v>
       </c>
       <c r="F306" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G306" t="n">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="H306" t="n">
         <v>0</v>
@@ -10253,10 +10253,10 @@
         <v>41</v>
       </c>
       <c r="F307" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G307" t="n">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="H307" t="n">
         <v>0</v>
@@ -10282,13 +10282,13 @@
         <v>41</v>
       </c>
       <c r="E308" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F308" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G308" t="n">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="H308" t="n">
         <v>0</v>
@@ -10314,13 +10314,13 @@
         <v>41</v>
       </c>
       <c r="E309" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F309" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G309" t="n">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="H309" t="n">
         <v>0</v>
@@ -10349,10 +10349,10 @@
         <v>42</v>
       </c>
       <c r="F310" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G310" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H310" t="n">
         <v>0</v>
@@ -10381,10 +10381,10 @@
         <v>42</v>
       </c>
       <c r="F311" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G311" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H311" t="n">
         <v>0</v>
@@ -10413,10 +10413,10 @@
         <v>42</v>
       </c>
       <c r="F312" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G312" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H312" t="n">
         <v>0</v>
@@ -10445,10 +10445,10 @@
         <v>42</v>
       </c>
       <c r="F313" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G313" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H313" t="n">
         <v>0</v>
@@ -10477,10 +10477,10 @@
         <v>42</v>
       </c>
       <c r="F314" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G314" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H314" t="n">
         <v>0</v>
@@ -10509,10 +10509,10 @@
         <v>42</v>
       </c>
       <c r="F315" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G315" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H315" t="n">
         <v>0</v>
@@ -10541,10 +10541,10 @@
         <v>42</v>
       </c>
       <c r="F316" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G316" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H316" t="n">
         <v>0</v>
@@ -10573,10 +10573,10 @@
         <v>42</v>
       </c>
       <c r="F317" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G317" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H317" t="n">
         <v>0</v>
@@ -10605,10 +10605,10 @@
         <v>42</v>
       </c>
       <c r="F318" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G318" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H318" t="n">
         <v>0</v>
@@ -10637,10 +10637,10 @@
         <v>42</v>
       </c>
       <c r="F319" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G319" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H319" t="n">
         <v>0</v>
@@ -10669,10 +10669,10 @@
         <v>42</v>
       </c>
       <c r="F320" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G320" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H320" t="n">
         <v>0</v>
@@ -10701,10 +10701,10 @@
         <v>42</v>
       </c>
       <c r="F321" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G321" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H321" t="n">
         <v>0</v>
@@ -10733,10 +10733,10 @@
         <v>42</v>
       </c>
       <c r="F322" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G322" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H322" t="n">
         <v>0</v>
@@ -10765,10 +10765,10 @@
         <v>42</v>
       </c>
       <c r="F323" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G323" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="H323" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
ultimas adecuaciones, agrupación de turnos >7 hrs para mayor penalizacion
</commit_message>
<xml_diff>
--- a/Result/CoberturaFinal.xlsx
+++ b/Result/CoberturaFinal.xlsx
@@ -938,16 +938,16 @@
         <v>12</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="F16" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="G16" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -970,16 +970,16 @@
         <v>18</v>
       </c>
       <c r="E17" t="n">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="F17" t="n">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18">
@@ -1002,13 +1002,13 @@
         <v>380</v>
       </c>
       <c r="E18" t="n">
-        <v>183</v>
+        <v>123</v>
       </c>
       <c r="F18" t="n">
-        <v>183</v>
+        <v>123</v>
       </c>
       <c r="G18" t="n">
-        <v>197</v>
+        <v>257</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -1034,13 +1034,13 @@
         <v>400</v>
       </c>
       <c r="E19" t="n">
-        <v>279</v>
+        <v>153</v>
       </c>
       <c r="F19" t="n">
-        <v>279</v>
+        <v>153</v>
       </c>
       <c r="G19" t="n">
-        <v>121</v>
+        <v>247</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -1066,13 +1066,13 @@
         <v>416</v>
       </c>
       <c r="E20" t="n">
-        <v>363</v>
+        <v>248</v>
       </c>
       <c r="F20" t="n">
-        <v>363</v>
+        <v>248</v>
       </c>
       <c r="G20" t="n">
-        <v>53</v>
+        <v>168</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -1098,13 +1098,13 @@
         <v>440</v>
       </c>
       <c r="E21" t="n">
-        <v>393</v>
+        <v>298</v>
       </c>
       <c r="F21" t="n">
-        <v>393</v>
+        <v>298</v>
       </c>
       <c r="G21" t="n">
-        <v>47</v>
+        <v>142</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1130,13 +1130,13 @@
         <v>463</v>
       </c>
       <c r="E22" t="n">
-        <v>403</v>
+        <v>366</v>
       </c>
       <c r="F22" t="n">
-        <v>403</v>
+        <v>366</v>
       </c>
       <c r="G22" t="n">
-        <v>60</v>
+        <v>97</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1162,13 +1162,13 @@
         <v>463</v>
       </c>
       <c r="E23" t="n">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="F23" t="n">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="G23" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1194,13 +1194,13 @@
         <v>465</v>
       </c>
       <c r="E24" t="n">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="F24" t="n">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="G24" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1226,13 +1226,13 @@
         <v>501</v>
       </c>
       <c r="E25" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F25" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G25" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1258,13 +1258,13 @@
         <v>501</v>
       </c>
       <c r="E26" t="n">
-        <v>343</v>
+        <v>388</v>
       </c>
       <c r="F26" t="n">
-        <v>343</v>
+        <v>388</v>
       </c>
       <c r="G26" t="n">
-        <v>158</v>
+        <v>113</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1290,13 +1290,13 @@
         <v>501</v>
       </c>
       <c r="E27" t="n">
-        <v>382</v>
+        <v>418</v>
       </c>
       <c r="F27" t="n">
-        <v>382</v>
+        <v>418</v>
       </c>
       <c r="G27" t="n">
-        <v>119</v>
+        <v>83</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1482,13 +1482,13 @@
         <v>497</v>
       </c>
       <c r="E33" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F33" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G33" t="n">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -1514,13 +1514,13 @@
         <v>488</v>
       </c>
       <c r="E34" t="n">
-        <v>418</v>
+        <v>343</v>
       </c>
       <c r="F34" t="n">
-        <v>418</v>
+        <v>343</v>
       </c>
       <c r="G34" t="n">
-        <v>70</v>
+        <v>145</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -1546,13 +1546,13 @@
         <v>472</v>
       </c>
       <c r="E35" t="n">
-        <v>415</v>
+        <v>280</v>
       </c>
       <c r="F35" t="n">
-        <v>415</v>
+        <v>280</v>
       </c>
       <c r="G35" t="n">
-        <v>57</v>
+        <v>192</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -1578,13 +1578,13 @@
         <v>449</v>
       </c>
       <c r="E36" t="n">
-        <v>325</v>
+        <v>220</v>
       </c>
       <c r="F36" t="n">
-        <v>325</v>
+        <v>220</v>
       </c>
       <c r="G36" t="n">
-        <v>124</v>
+        <v>229</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -1610,16 +1610,16 @@
         <v>121</v>
       </c>
       <c r="E37" t="n">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="F37" t="n">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="38">
@@ -1674,13 +1674,13 @@
         <v>85</v>
       </c>
       <c r="E39" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="F39" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="G39" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -1706,13 +1706,13 @@
         <v>60</v>
       </c>
       <c r="E40" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="F40" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="G40" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -1738,13 +1738,13 @@
         <v>37</v>
       </c>
       <c r="E41" t="n">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="F41" t="n">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="G41" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -1770,13 +1770,13 @@
         <v>37</v>
       </c>
       <c r="E42" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F42" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G42" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -1802,13 +1802,13 @@
         <v>37</v>
       </c>
       <c r="E43" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F43" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G43" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -2474,16 +2474,16 @@
         <v>11</v>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="F64" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="G64" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="65">
@@ -2506,16 +2506,16 @@
         <v>17</v>
       </c>
       <c r="E65" t="n">
-        <v>17</v>
+        <v>90</v>
       </c>
       <c r="F65" t="n">
-        <v>17</v>
+        <v>90</v>
       </c>
       <c r="G65" t="n">
         <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
     </row>
     <row r="66">
@@ -2538,13 +2538,13 @@
         <v>360</v>
       </c>
       <c r="E66" t="n">
-        <v>197</v>
+        <v>135</v>
       </c>
       <c r="F66" t="n">
-        <v>197</v>
+        <v>135</v>
       </c>
       <c r="G66" t="n">
-        <v>163</v>
+        <v>225</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
@@ -2570,13 +2570,13 @@
         <v>374</v>
       </c>
       <c r="E67" t="n">
-        <v>287</v>
+        <v>165</v>
       </c>
       <c r="F67" t="n">
-        <v>287</v>
+        <v>165</v>
       </c>
       <c r="G67" t="n">
-        <v>87</v>
+        <v>209</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -2602,13 +2602,13 @@
         <v>388</v>
       </c>
       <c r="E68" t="n">
-        <v>382</v>
+        <v>260</v>
       </c>
       <c r="F68" t="n">
-        <v>382</v>
+        <v>260</v>
       </c>
       <c r="G68" t="n">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
@@ -2634,13 +2634,13 @@
         <v>407</v>
       </c>
       <c r="E69" t="n">
-        <v>407</v>
+        <v>310</v>
       </c>
       <c r="F69" t="n">
-        <v>407</v>
+        <v>310</v>
       </c>
       <c r="G69" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
@@ -2666,13 +2666,13 @@
         <v>422</v>
       </c>
       <c r="E70" t="n">
-        <v>407</v>
+        <v>369</v>
       </c>
       <c r="F70" t="n">
-        <v>407</v>
+        <v>369</v>
       </c>
       <c r="G70" t="n">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="H70" t="n">
         <v>0</v>
@@ -2698,13 +2698,13 @@
         <v>423</v>
       </c>
       <c r="E71" t="n">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="F71" t="n">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="G71" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="H71" t="n">
         <v>0</v>
@@ -2730,13 +2730,13 @@
         <v>427</v>
       </c>
       <c r="E72" t="n">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="F72" t="n">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="G72" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="H72" t="n">
         <v>0</v>
@@ -2762,13 +2762,13 @@
         <v>457</v>
       </c>
       <c r="E73" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F73" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G73" t="n">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="H73" t="n">
         <v>0</v>
@@ -2794,13 +2794,13 @@
         <v>457</v>
       </c>
       <c r="E74" t="n">
-        <v>328</v>
+        <v>388</v>
       </c>
       <c r="F74" t="n">
-        <v>328</v>
+        <v>388</v>
       </c>
       <c r="G74" t="n">
-        <v>129</v>
+        <v>69</v>
       </c>
       <c r="H74" t="n">
         <v>0</v>
@@ -2826,13 +2826,13 @@
         <v>457</v>
       </c>
       <c r="E75" t="n">
-        <v>373</v>
+        <v>418</v>
       </c>
       <c r="F75" t="n">
-        <v>373</v>
+        <v>418</v>
       </c>
       <c r="G75" t="n">
-        <v>84</v>
+        <v>39</v>
       </c>
       <c r="H75" t="n">
         <v>0</v>
@@ -3018,13 +3018,13 @@
         <v>453</v>
       </c>
       <c r="E81" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F81" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G81" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="H81" t="n">
         <v>0</v>
@@ -3050,13 +3050,13 @@
         <v>442</v>
       </c>
       <c r="E82" t="n">
-        <v>418</v>
+        <v>343</v>
       </c>
       <c r="F82" t="n">
-        <v>418</v>
+        <v>343</v>
       </c>
       <c r="G82" t="n">
-        <v>24</v>
+        <v>99</v>
       </c>
       <c r="H82" t="n">
         <v>0</v>
@@ -3082,13 +3082,13 @@
         <v>427</v>
       </c>
       <c r="E83" t="n">
-        <v>416</v>
+        <v>268</v>
       </c>
       <c r="F83" t="n">
-        <v>416</v>
+        <v>268</v>
       </c>
       <c r="G83" t="n">
-        <v>11</v>
+        <v>159</v>
       </c>
       <c r="H83" t="n">
         <v>0</v>
@@ -3114,13 +3114,13 @@
         <v>402</v>
       </c>
       <c r="E84" t="n">
-        <v>326</v>
+        <v>208</v>
       </c>
       <c r="F84" t="n">
-        <v>326</v>
+        <v>208</v>
       </c>
       <c r="G84" t="n">
-        <v>76</v>
+        <v>194</v>
       </c>
       <c r="H84" t="n">
         <v>0</v>
@@ -3146,16 +3146,16 @@
         <v>95</v>
       </c>
       <c r="E85" t="n">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F85" t="n">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="G85" t="n">
         <v>0</v>
       </c>
       <c r="H85" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="86">
@@ -3178,16 +3178,16 @@
         <v>81</v>
       </c>
       <c r="E86" t="n">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="F86" t="n">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="G86" t="n">
         <v>0</v>
       </c>
       <c r="H86" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="87">
@@ -3210,13 +3210,13 @@
         <v>69</v>
       </c>
       <c r="E87" t="n">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="F87" t="n">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="G87" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="H87" t="n">
         <v>0</v>
@@ -3242,13 +3242,13 @@
         <v>48</v>
       </c>
       <c r="E88" t="n">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="F88" t="n">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="G88" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H88" t="n">
         <v>0</v>
@@ -3274,13 +3274,13 @@
         <v>34</v>
       </c>
       <c r="E89" t="n">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F89" t="n">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="G89" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="H89" t="n">
         <v>0</v>
@@ -3306,13 +3306,13 @@
         <v>34</v>
       </c>
       <c r="E90" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F90" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="G90" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H90" t="n">
         <v>0</v>
@@ -3338,13 +3338,13 @@
         <v>32</v>
       </c>
       <c r="E91" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F91" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="G91" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="H91" t="n">
         <v>0</v>
@@ -4010,16 +4010,16 @@
         <v>11</v>
       </c>
       <c r="E112" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F112" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="G112" t="n">
         <v>0</v>
       </c>
       <c r="H112" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="113">
@@ -4042,16 +4042,16 @@
         <v>17</v>
       </c>
       <c r="E113" t="n">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="F113" t="n">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="G113" t="n">
         <v>0</v>
       </c>
       <c r="H113" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
     </row>
     <row r="114">
@@ -4074,13 +4074,13 @@
         <v>319</v>
       </c>
       <c r="E114" t="n">
-        <v>213</v>
+        <v>131</v>
       </c>
       <c r="F114" t="n">
-        <v>213</v>
+        <v>131</v>
       </c>
       <c r="G114" t="n">
-        <v>106</v>
+        <v>188</v>
       </c>
       <c r="H114" t="n">
         <v>0</v>
@@ -4106,13 +4106,13 @@
         <v>336</v>
       </c>
       <c r="E115" t="n">
-        <v>310</v>
+        <v>168</v>
       </c>
       <c r="F115" t="n">
-        <v>310</v>
+        <v>168</v>
       </c>
       <c r="G115" t="n">
-        <v>26</v>
+        <v>168</v>
       </c>
       <c r="H115" t="n">
         <v>0</v>
@@ -4138,13 +4138,13 @@
         <v>347</v>
       </c>
       <c r="E116" t="n">
-        <v>347</v>
+        <v>263</v>
       </c>
       <c r="F116" t="n">
-        <v>347</v>
+        <v>263</v>
       </c>
       <c r="G116" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="H116" t="n">
         <v>0</v>
@@ -4170,13 +4170,13 @@
         <v>364</v>
       </c>
       <c r="E117" t="n">
-        <v>364</v>
+        <v>318</v>
       </c>
       <c r="F117" t="n">
-        <v>364</v>
+        <v>318</v>
       </c>
       <c r="G117" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="H117" t="n">
         <v>0</v>
@@ -4202,13 +4202,13 @@
         <v>385</v>
       </c>
       <c r="E118" t="n">
-        <v>385</v>
+        <v>369</v>
       </c>
       <c r="F118" t="n">
-        <v>385</v>
+        <v>369</v>
       </c>
       <c r="G118" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H118" t="n">
         <v>0</v>
@@ -4298,13 +4298,13 @@
         <v>413</v>
       </c>
       <c r="E121" t="n">
-        <v>413</v>
+        <v>403</v>
       </c>
       <c r="F121" t="n">
-        <v>413</v>
+        <v>403</v>
       </c>
       <c r="G121" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H121" t="n">
         <v>0</v>
@@ -4330,13 +4330,13 @@
         <v>411</v>
       </c>
       <c r="E122" t="n">
-        <v>338</v>
+        <v>381</v>
       </c>
       <c r="F122" t="n">
-        <v>338</v>
+        <v>381</v>
       </c>
       <c r="G122" t="n">
-        <v>73</v>
+        <v>30</v>
       </c>
       <c r="H122" t="n">
         <v>0</v>
@@ -4362,13 +4362,13 @@
         <v>411</v>
       </c>
       <c r="E123" t="n">
-        <v>383</v>
+        <v>411</v>
       </c>
       <c r="F123" t="n">
-        <v>383</v>
+        <v>411</v>
       </c>
       <c r="G123" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="H123" t="n">
         <v>0</v>
@@ -4426,13 +4426,13 @@
         <v>413</v>
       </c>
       <c r="E125" t="n">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="F125" t="n">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="G125" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H125" t="n">
         <v>0</v>
@@ -4490,13 +4490,13 @@
         <v>411</v>
       </c>
       <c r="E127" t="n">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="F127" t="n">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="G127" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H127" t="n">
         <v>0</v>
@@ -4554,13 +4554,13 @@
         <v>409</v>
       </c>
       <c r="E129" t="n">
-        <v>409</v>
+        <v>394</v>
       </c>
       <c r="F129" t="n">
-        <v>409</v>
+        <v>394</v>
       </c>
       <c r="G129" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H129" t="n">
         <v>0</v>
@@ -4586,13 +4586,13 @@
         <v>398</v>
       </c>
       <c r="E130" t="n">
-        <v>398</v>
+        <v>329</v>
       </c>
       <c r="F130" t="n">
-        <v>398</v>
+        <v>329</v>
       </c>
       <c r="G130" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="H130" t="n">
         <v>0</v>
@@ -4618,13 +4618,13 @@
         <v>381</v>
       </c>
       <c r="E131" t="n">
-        <v>381</v>
+        <v>265</v>
       </c>
       <c r="F131" t="n">
-        <v>381</v>
+        <v>265</v>
       </c>
       <c r="G131" t="n">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="H131" t="n">
         <v>0</v>
@@ -4650,13 +4650,13 @@
         <v>359</v>
       </c>
       <c r="E132" t="n">
-        <v>300</v>
+        <v>201</v>
       </c>
       <c r="F132" t="n">
-        <v>300</v>
+        <v>201</v>
       </c>
       <c r="G132" t="n">
-        <v>59</v>
+        <v>158</v>
       </c>
       <c r="H132" t="n">
         <v>0</v>
@@ -4682,16 +4682,16 @@
         <v>95</v>
       </c>
       <c r="E133" t="n">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="F133" t="n">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="G133" t="n">
         <v>0</v>
       </c>
       <c r="H133" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="134">
@@ -4746,13 +4746,13 @@
         <v>66</v>
       </c>
       <c r="E135" t="n">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="F135" t="n">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="G135" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H135" t="n">
         <v>0</v>
@@ -4778,13 +4778,13 @@
         <v>48</v>
       </c>
       <c r="E136" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="F136" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="G136" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H136" t="n">
         <v>0</v>
@@ -5514,13 +5514,13 @@
         <v>1</v>
       </c>
       <c r="E159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G159" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H159" t="n">
         <v>0</v>
@@ -5546,16 +5546,16 @@
         <v>7</v>
       </c>
       <c r="E160" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="F160" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="G160" t="n">
         <v>0</v>
       </c>
       <c r="H160" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="161">
@@ -5578,16 +5578,16 @@
         <v>10</v>
       </c>
       <c r="E161" t="n">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="F161" t="n">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="G161" t="n">
         <v>0</v>
       </c>
       <c r="H161" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="162">
@@ -5610,13 +5610,13 @@
         <v>362</v>
       </c>
       <c r="E162" t="n">
-        <v>205</v>
+        <v>86</v>
       </c>
       <c r="F162" t="n">
-        <v>205</v>
+        <v>86</v>
       </c>
       <c r="G162" t="n">
-        <v>157</v>
+        <v>276</v>
       </c>
       <c r="H162" t="n">
         <v>0</v>
@@ -5642,13 +5642,13 @@
         <v>376</v>
       </c>
       <c r="E163" t="n">
-        <v>325</v>
+        <v>131</v>
       </c>
       <c r="F163" t="n">
-        <v>325</v>
+        <v>131</v>
       </c>
       <c r="G163" t="n">
-        <v>51</v>
+        <v>245</v>
       </c>
       <c r="H163" t="n">
         <v>0</v>
@@ -5674,13 +5674,13 @@
         <v>391</v>
       </c>
       <c r="E164" t="n">
-        <v>356</v>
+        <v>251</v>
       </c>
       <c r="F164" t="n">
-        <v>356</v>
+        <v>251</v>
       </c>
       <c r="G164" t="n">
-        <v>35</v>
+        <v>140</v>
       </c>
       <c r="H164" t="n">
         <v>0</v>
@@ -5706,13 +5706,13 @@
         <v>408</v>
       </c>
       <c r="E165" t="n">
-        <v>386</v>
+        <v>301</v>
       </c>
       <c r="F165" t="n">
-        <v>386</v>
+        <v>301</v>
       </c>
       <c r="G165" t="n">
-        <v>22</v>
+        <v>107</v>
       </c>
       <c r="H165" t="n">
         <v>0</v>
@@ -5738,13 +5738,13 @@
         <v>428</v>
       </c>
       <c r="E166" t="n">
-        <v>401</v>
+        <v>381</v>
       </c>
       <c r="F166" t="n">
-        <v>401</v>
+        <v>381</v>
       </c>
       <c r="G166" t="n">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="H166" t="n">
         <v>0</v>
@@ -5770,13 +5770,13 @@
         <v>428</v>
       </c>
       <c r="E167" t="n">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="F167" t="n">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="G167" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H167" t="n">
         <v>0</v>
@@ -5802,13 +5802,13 @@
         <v>429</v>
       </c>
       <c r="E168" t="n">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="F168" t="n">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="G168" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="H168" t="n">
         <v>0</v>
@@ -5866,13 +5866,13 @@
         <v>454</v>
       </c>
       <c r="E170" t="n">
-        <v>328</v>
+        <v>388</v>
       </c>
       <c r="F170" t="n">
-        <v>328</v>
+        <v>388</v>
       </c>
       <c r="G170" t="n">
-        <v>126</v>
+        <v>66</v>
       </c>
       <c r="H170" t="n">
         <v>0</v>
@@ -5898,13 +5898,13 @@
         <v>454</v>
       </c>
       <c r="E171" t="n">
-        <v>343</v>
+        <v>373</v>
       </c>
       <c r="F171" t="n">
-        <v>343</v>
+        <v>373</v>
       </c>
       <c r="G171" t="n">
-        <v>111</v>
+        <v>81</v>
       </c>
       <c r="H171" t="n">
         <v>0</v>
@@ -5930,13 +5930,13 @@
         <v>454</v>
       </c>
       <c r="E172" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F172" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="G172" t="n">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="H172" t="n">
         <v>0</v>
@@ -5962,13 +5962,13 @@
         <v>454</v>
       </c>
       <c r="E173" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="F173" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="G173" t="n">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="H173" t="n">
         <v>0</v>
@@ -5994,13 +5994,13 @@
         <v>451</v>
       </c>
       <c r="E174" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="F174" t="n">
-        <v>418</v>
+        <v>388</v>
       </c>
       <c r="G174" t="n">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="H174" t="n">
         <v>0</v>
@@ -6122,13 +6122,13 @@
         <v>442</v>
       </c>
       <c r="E178" t="n">
-        <v>418</v>
+        <v>357</v>
       </c>
       <c r="F178" t="n">
-        <v>418</v>
+        <v>357</v>
       </c>
       <c r="G178" t="n">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="H178" t="n">
         <v>0</v>
@@ -6154,13 +6154,13 @@
         <v>430</v>
       </c>
       <c r="E179" t="n">
-        <v>396</v>
+        <v>302</v>
       </c>
       <c r="F179" t="n">
-        <v>396</v>
+        <v>302</v>
       </c>
       <c r="G179" t="n">
-        <v>34</v>
+        <v>128</v>
       </c>
       <c r="H179" t="n">
         <v>0</v>
@@ -6186,13 +6186,13 @@
         <v>390</v>
       </c>
       <c r="E180" t="n">
-        <v>318</v>
+        <v>227</v>
       </c>
       <c r="F180" t="n">
-        <v>318</v>
+        <v>227</v>
       </c>
       <c r="G180" t="n">
-        <v>72</v>
+        <v>163</v>
       </c>
       <c r="H180" t="n">
         <v>0</v>
@@ -6218,16 +6218,16 @@
         <v>91</v>
       </c>
       <c r="E181" t="n">
-        <v>91</v>
+        <v>167</v>
       </c>
       <c r="F181" t="n">
-        <v>91</v>
+        <v>167</v>
       </c>
       <c r="G181" t="n">
         <v>0</v>
       </c>
       <c r="H181" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
     </row>
     <row r="182">
@@ -6250,16 +6250,16 @@
         <v>74</v>
       </c>
       <c r="E182" t="n">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="F182" t="n">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="G182" t="n">
         <v>0</v>
       </c>
       <c r="H182" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="183">
@@ -6314,13 +6314,13 @@
         <v>45</v>
       </c>
       <c r="E184" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="F184" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="G184" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="H184" t="n">
         <v>0</v>
@@ -6346,13 +6346,13 @@
         <v>27</v>
       </c>
       <c r="E185" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F185" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G185" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H185" t="n">
         <v>0</v>
@@ -6378,13 +6378,13 @@
         <v>27</v>
       </c>
       <c r="E186" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F186" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G186" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="H186" t="n">
         <v>0</v>
@@ -6410,13 +6410,13 @@
         <v>26</v>
       </c>
       <c r="E187" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F187" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G187" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H187" t="n">
         <v>0</v>
@@ -7082,16 +7082,16 @@
         <v>6</v>
       </c>
       <c r="E208" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F208" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="G208" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H208" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="209">
@@ -7114,16 +7114,16 @@
         <v>12</v>
       </c>
       <c r="E209" t="n">
-        <v>12</v>
+        <v>86</v>
       </c>
       <c r="F209" t="n">
-        <v>12</v>
+        <v>86</v>
       </c>
       <c r="G209" t="n">
         <v>0</v>
       </c>
       <c r="H209" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
     </row>
     <row r="210">
@@ -7146,13 +7146,13 @@
         <v>367</v>
       </c>
       <c r="E210" t="n">
-        <v>187</v>
+        <v>131</v>
       </c>
       <c r="F210" t="n">
-        <v>97</v>
+        <v>131</v>
       </c>
       <c r="G210" t="n">
-        <v>270</v>
+        <v>236</v>
       </c>
       <c r="H210" t="n">
         <v>0</v>
@@ -7178,13 +7178,13 @@
         <v>385</v>
       </c>
       <c r="E211" t="n">
-        <v>286</v>
+        <v>161</v>
       </c>
       <c r="F211" t="n">
-        <v>118</v>
+        <v>161</v>
       </c>
       <c r="G211" t="n">
-        <v>267</v>
+        <v>224</v>
       </c>
       <c r="H211" t="n">
         <v>0</v>
@@ -7210,13 +7210,13 @@
         <v>402</v>
       </c>
       <c r="E212" t="n">
-        <v>376</v>
+        <v>256</v>
       </c>
       <c r="F212" t="n">
-        <v>208</v>
+        <v>256</v>
       </c>
       <c r="G212" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="H212" t="n">
         <v>0</v>
@@ -7242,13 +7242,13 @@
         <v>422</v>
       </c>
       <c r="E213" t="n">
-        <v>406</v>
+        <v>306</v>
       </c>
       <c r="F213" t="n">
-        <v>238</v>
+        <v>306</v>
       </c>
       <c r="G213" t="n">
-        <v>184</v>
+        <v>116</v>
       </c>
       <c r="H213" t="n">
         <v>0</v>
@@ -7274,13 +7274,13 @@
         <v>438</v>
       </c>
       <c r="E214" t="n">
-        <v>406</v>
+        <v>368</v>
       </c>
       <c r="F214" t="n">
-        <v>238</v>
+        <v>368</v>
       </c>
       <c r="G214" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="H214" t="n">
         <v>0</v>
@@ -7306,13 +7306,13 @@
         <v>438</v>
       </c>
       <c r="E215" t="n">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="F215" t="n">
-        <v>238</v>
+        <v>413</v>
       </c>
       <c r="G215" t="n">
-        <v>200</v>
+        <v>25</v>
       </c>
       <c r="H215" t="n">
         <v>0</v>
@@ -7338,13 +7338,13 @@
         <v>440</v>
       </c>
       <c r="E216" t="n">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="F216" t="n">
-        <v>238</v>
+        <v>413</v>
       </c>
       <c r="G216" t="n">
-        <v>202</v>
+        <v>27</v>
       </c>
       <c r="H216" t="n">
         <v>0</v>
@@ -7370,13 +7370,13 @@
         <v>472</v>
       </c>
       <c r="E217" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F217" t="n">
-        <v>250</v>
+        <v>403</v>
       </c>
       <c r="G217" t="n">
-        <v>222</v>
+        <v>69</v>
       </c>
       <c r="H217" t="n">
         <v>0</v>
@@ -7402,13 +7402,13 @@
         <v>472</v>
       </c>
       <c r="E218" t="n">
-        <v>363</v>
+        <v>388</v>
       </c>
       <c r="F218" t="n">
-        <v>195</v>
+        <v>388</v>
       </c>
       <c r="G218" t="n">
-        <v>277</v>
+        <v>84</v>
       </c>
       <c r="H218" t="n">
         <v>0</v>
@@ -7434,13 +7434,13 @@
         <v>472</v>
       </c>
       <c r="E219" t="n">
-        <v>405</v>
+        <v>418</v>
       </c>
       <c r="F219" t="n">
-        <v>237</v>
+        <v>418</v>
       </c>
       <c r="G219" t="n">
-        <v>235</v>
+        <v>54</v>
       </c>
       <c r="H219" t="n">
         <v>0</v>
@@ -7469,10 +7469,10 @@
         <v>418</v>
       </c>
       <c r="F220" t="n">
-        <v>250</v>
+        <v>418</v>
       </c>
       <c r="G220" t="n">
-        <v>223</v>
+        <v>55</v>
       </c>
       <c r="H220" t="n">
         <v>0</v>
@@ -7501,10 +7501,10 @@
         <v>418</v>
       </c>
       <c r="F221" t="n">
-        <v>250</v>
+        <v>418</v>
       </c>
       <c r="G221" t="n">
-        <v>223</v>
+        <v>55</v>
       </c>
       <c r="H221" t="n">
         <v>0</v>
@@ -7533,10 +7533,10 @@
         <v>418</v>
       </c>
       <c r="F222" t="n">
-        <v>250</v>
+        <v>418</v>
       </c>
       <c r="G222" t="n">
-        <v>222</v>
+        <v>54</v>
       </c>
       <c r="H222" t="n">
         <v>0</v>
@@ -7565,10 +7565,10 @@
         <v>418</v>
       </c>
       <c r="F223" t="n">
-        <v>250</v>
+        <v>418</v>
       </c>
       <c r="G223" t="n">
-        <v>221</v>
+        <v>53</v>
       </c>
       <c r="H223" t="n">
         <v>0</v>
@@ -7597,10 +7597,10 @@
         <v>418</v>
       </c>
       <c r="F224" t="n">
-        <v>250</v>
+        <v>418</v>
       </c>
       <c r="G224" t="n">
-        <v>218</v>
+        <v>50</v>
       </c>
       <c r="H224" t="n">
         <v>0</v>
@@ -7626,13 +7626,13 @@
         <v>462</v>
       </c>
       <c r="E225" t="n">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="F225" t="n">
-        <v>250</v>
+        <v>403</v>
       </c>
       <c r="G225" t="n">
-        <v>212</v>
+        <v>59</v>
       </c>
       <c r="H225" t="n">
         <v>0</v>
@@ -7658,13 +7658,13 @@
         <v>438</v>
       </c>
       <c r="E226" t="n">
-        <v>418</v>
+        <v>343</v>
       </c>
       <c r="F226" t="n">
-        <v>250</v>
+        <v>343</v>
       </c>
       <c r="G226" t="n">
-        <v>188</v>
+        <v>95</v>
       </c>
       <c r="H226" t="n">
         <v>0</v>
@@ -7690,13 +7690,13 @@
         <v>431</v>
       </c>
       <c r="E227" t="n">
-        <v>388</v>
+        <v>272</v>
       </c>
       <c r="F227" t="n">
-        <v>250</v>
+        <v>272</v>
       </c>
       <c r="G227" t="n">
-        <v>181</v>
+        <v>159</v>
       </c>
       <c r="H227" t="n">
         <v>0</v>
@@ -7722,13 +7722,13 @@
         <v>216</v>
       </c>
       <c r="E228" t="n">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="F228" t="n">
-        <v>168</v>
+        <v>212</v>
       </c>
       <c r="G228" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="H228" t="n">
         <v>0</v>
@@ -7754,16 +7754,16 @@
         <v>105</v>
       </c>
       <c r="E229" t="n">
-        <v>105</v>
+        <v>137</v>
       </c>
       <c r="F229" t="n">
-        <v>105</v>
+        <v>137</v>
       </c>
       <c r="G229" t="n">
         <v>0</v>
       </c>
       <c r="H229" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
     </row>
     <row r="230">
@@ -7786,16 +7786,16 @@
         <v>87</v>
       </c>
       <c r="E230" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F230" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="G230" t="n">
         <v>0</v>
       </c>
       <c r="H230" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="231">
@@ -7818,13 +7818,13 @@
         <v>73</v>
       </c>
       <c r="E231" t="n">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="F231" t="n">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="G231" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="H231" t="n">
         <v>0</v>
@@ -7850,13 +7850,13 @@
         <v>52</v>
       </c>
       <c r="E232" t="n">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="F232" t="n">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="G232" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="H232" t="n">
         <v>0</v>
@@ -7882,13 +7882,13 @@
         <v>35</v>
       </c>
       <c r="E233" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="F233" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G233" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="H233" t="n">
         <v>0</v>
@@ -7914,13 +7914,13 @@
         <v>35</v>
       </c>
       <c r="E234" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F234" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G234" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H234" t="n">
         <v>0</v>
@@ -7946,13 +7946,13 @@
         <v>34</v>
       </c>
       <c r="E235" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F235" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G235" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H235" t="n">
         <v>0</v>
@@ -8685,10 +8685,10 @@
         <v>204</v>
       </c>
       <c r="F258" t="n">
-        <v>144</v>
+        <v>204</v>
       </c>
       <c r="G258" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H258" t="n">
         <v>0</v>
@@ -8717,10 +8717,10 @@
         <v>204</v>
       </c>
       <c r="F259" t="n">
-        <v>144</v>
+        <v>204</v>
       </c>
       <c r="G259" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H259" t="n">
         <v>0</v>
@@ -8749,10 +8749,10 @@
         <v>206</v>
       </c>
       <c r="F260" t="n">
-        <v>146</v>
+        <v>206</v>
       </c>
       <c r="G260" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H260" t="n">
         <v>0</v>
@@ -8781,10 +8781,10 @@
         <v>207</v>
       </c>
       <c r="F261" t="n">
-        <v>147</v>
+        <v>207</v>
       </c>
       <c r="G261" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H261" t="n">
         <v>0</v>
@@ -8813,10 +8813,10 @@
         <v>208</v>
       </c>
       <c r="F262" t="n">
-        <v>148</v>
+        <v>208</v>
       </c>
       <c r="G262" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H262" t="n">
         <v>0</v>
@@ -8845,10 +8845,10 @@
         <v>208</v>
       </c>
       <c r="F263" t="n">
-        <v>148</v>
+        <v>208</v>
       </c>
       <c r="G263" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H263" t="n">
         <v>0</v>
@@ -8877,10 +8877,10 @@
         <v>209</v>
       </c>
       <c r="F264" t="n">
-        <v>149</v>
+        <v>209</v>
       </c>
       <c r="G264" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H264" t="n">
         <v>0</v>
@@ -8909,10 +8909,10 @@
         <v>209</v>
       </c>
       <c r="F265" t="n">
-        <v>149</v>
+        <v>209</v>
       </c>
       <c r="G265" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H265" t="n">
         <v>0</v>
@@ -8938,13 +8938,13 @@
         <v>209</v>
       </c>
       <c r="E266" t="n">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="F266" t="n">
-        <v>149</v>
+        <v>198</v>
       </c>
       <c r="G266" t="n">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="H266" t="n">
         <v>0</v>
@@ -8973,10 +8973,10 @@
         <v>209</v>
       </c>
       <c r="F267" t="n">
-        <v>149</v>
+        <v>209</v>
       </c>
       <c r="G267" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H267" t="n">
         <v>0</v>
@@ -9005,10 +9005,10 @@
         <v>209</v>
       </c>
       <c r="F268" t="n">
-        <v>149</v>
+        <v>209</v>
       </c>
       <c r="G268" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H268" t="n">
         <v>0</v>
@@ -9037,10 +9037,10 @@
         <v>208</v>
       </c>
       <c r="F269" t="n">
-        <v>148</v>
+        <v>208</v>
       </c>
       <c r="G269" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H269" t="n">
         <v>0</v>
@@ -9069,10 +9069,10 @@
         <v>205</v>
       </c>
       <c r="F270" t="n">
-        <v>145</v>
+        <v>205</v>
       </c>
       <c r="G270" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H270" t="n">
         <v>0</v>
@@ -9098,13 +9098,13 @@
         <v>205</v>
       </c>
       <c r="E271" t="n">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F271" t="n">
-        <v>145</v>
+        <v>204</v>
       </c>
       <c r="G271" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="H271" t="n">
         <v>0</v>
@@ -9133,10 +9133,10 @@
         <v>201</v>
       </c>
       <c r="F272" t="n">
-        <v>141</v>
+        <v>201</v>
       </c>
       <c r="G272" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H272" t="n">
         <v>0</v>
@@ -9165,10 +9165,10 @@
         <v>201</v>
       </c>
       <c r="F273" t="n">
-        <v>141</v>
+        <v>201</v>
       </c>
       <c r="G273" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H273" t="n">
         <v>0</v>
@@ -9197,10 +9197,10 @@
         <v>198</v>
       </c>
       <c r="F274" t="n">
-        <v>138</v>
+        <v>198</v>
       </c>
       <c r="G274" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H274" t="n">
         <v>0</v>
@@ -9226,13 +9226,13 @@
         <v>198</v>
       </c>
       <c r="E275" t="n">
-        <v>198</v>
+        <v>172</v>
       </c>
       <c r="F275" t="n">
-        <v>138</v>
+        <v>172</v>
       </c>
       <c r="G275" t="n">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="H275" t="n">
         <v>0</v>
@@ -10221,10 +10221,10 @@
         <v>41</v>
       </c>
       <c r="F306" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="G306" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H306" t="n">
         <v>0</v>
@@ -10253,10 +10253,10 @@
         <v>41</v>
       </c>
       <c r="F307" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="G307" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H307" t="n">
         <v>0</v>
@@ -10285,10 +10285,10 @@
         <v>41</v>
       </c>
       <c r="F308" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="G308" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H308" t="n">
         <v>0</v>
@@ -10317,10 +10317,10 @@
         <v>41</v>
       </c>
       <c r="F309" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="G309" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H309" t="n">
         <v>0</v>
@@ -10349,10 +10349,10 @@
         <v>42</v>
       </c>
       <c r="F310" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G310" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H310" t="n">
         <v>0</v>
@@ -10381,10 +10381,10 @@
         <v>42</v>
       </c>
       <c r="F311" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G311" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H311" t="n">
         <v>0</v>
@@ -10413,10 +10413,10 @@
         <v>42</v>
       </c>
       <c r="F312" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G312" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H312" t="n">
         <v>0</v>
@@ -10445,10 +10445,10 @@
         <v>42</v>
       </c>
       <c r="F313" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G313" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H313" t="n">
         <v>0</v>
@@ -10477,10 +10477,10 @@
         <v>42</v>
       </c>
       <c r="F314" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G314" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H314" t="n">
         <v>0</v>
@@ -10509,10 +10509,10 @@
         <v>42</v>
       </c>
       <c r="F315" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G315" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H315" t="n">
         <v>0</v>
@@ -10541,10 +10541,10 @@
         <v>42</v>
       </c>
       <c r="F316" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G316" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H316" t="n">
         <v>0</v>
@@ -10573,10 +10573,10 @@
         <v>42</v>
       </c>
       <c r="F317" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G317" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H317" t="n">
         <v>0</v>
@@ -10605,10 +10605,10 @@
         <v>42</v>
       </c>
       <c r="F318" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G318" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H318" t="n">
         <v>0</v>
@@ -10637,10 +10637,10 @@
         <v>42</v>
       </c>
       <c r="F319" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G319" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H319" t="n">
         <v>0</v>
@@ -10669,10 +10669,10 @@
         <v>42</v>
       </c>
       <c r="F320" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G320" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H320" t="n">
         <v>0</v>
@@ -10701,10 +10701,10 @@
         <v>42</v>
       </c>
       <c r="F321" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G321" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H321" t="n">
         <v>0</v>
@@ -10733,10 +10733,10 @@
         <v>42</v>
       </c>
       <c r="F322" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G322" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H322" t="n">
         <v>0</v>
@@ -10765,10 +10765,10 @@
         <v>42</v>
       </c>
       <c r="F323" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G323" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H323" t="n">
         <v>0</v>

</xml_diff>